<commit_message>
Round 2 model: usage-tiered fleet battery EMI, Maruti strategic case
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtuctuJfT3uCJpQnU6kHYK
</commit_message>
<xml_diff>
--- a/Round2/Tour-e_TCO_Model_R2.xlsx
+++ b/Round2/Tour-e_TCO_Model_R2.xlsx
@@ -27,12 +27,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="0.00&quot;×&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot;×&quot;"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -144,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,11 +154,11 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -183,6 +184,7 @@
     <xf numFmtId="49" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -964,7 +966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1036,7 +1038,7 @@
       </c>
       <c r="B7" s="6">
         <f>Fleet_Economics!C7</f>
-        <v>0.9039999999999998</v>
+        <v>1.2239999999999993</v>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
@@ -1052,7 +1054,7 @@
       </c>
       <c r="B8" s="8" t="str">
         <f>TEXT(TCO!B30,"0.00")&amp;" / "&amp;TEXT(TCO!C30,"0.00")&amp;" / "&amp;TEXT(TCO!D30,"0.00")</f>
-        <v>8.86 / 7.73 / 7.13</v>
+        <v>8.86 / 7.33 / 7.13</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
@@ -1077,291 +1079,364 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>OWNER-DRIVER (60,000 km/yr)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Battery-EMI car vs Ertiga CNG: upfront price difference (₹ lakh)</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
+        <f>Fleet_Economics!C10</f>
+        <v>-1.5459919999999983</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Fleet_Economics</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>5-year saving per car, Tour-e outright (₹ lakh)</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>Fleet_Economics!D8</f>
+        <v>6.919999999999998</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Fleet_Economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Annual saving for a 1,000-car fleet, outright / EMI (₹ crore)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="str">
+        <f>TEXT(Fleet_Economics!D7*10,"0.0")&amp;" / "&amp;TEXT(Fleet_Economics!C7*10,"0.0")</f>
+        <v>13.8 / 12.2</v>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Fleet_Economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>OWNER-DRIVER (60,000 km/yr)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Gain per month vs CNG, Maruti driver hub charging – EMI (₹)</t>
         </is>
       </c>
-      <c r="B11" s="8">
+      <c r="B14" s="8">
         <f>Driver_Economics!C11</f>
         <v>5150.000000000007</v>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Driver_Economics</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Gain per month vs CNG, Maruti driver hub charging – outright (₹)</t>
         </is>
       </c>
-      <c r="B12" s="8">
+      <c r="B15" s="8">
         <f>Driver_Economics!D11</f>
         <v>5600.000000000007</v>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Driver_Economics</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Gain per month vs CNG with no hub (EMI / outright, ₹)</t>
         </is>
       </c>
-      <c r="B13" s="10" t="str">
+      <c r="B16" s="6" t="str">
         <f>Driver_Economics!E28</f>
         <v>1,400 / 1,850</v>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Driver_Economics</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>VEHICLE AND PRICE</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Ex-factory cost 2028 / 2035 (₹ lakh)</t>
         </is>
       </c>
-      <c r="B15" s="10" t="str">
+      <c r="B18" s="6" t="str">
         <f>TEXT(Cost_Price!$B$18,"0.00")&amp;" / "&amp;TEXT(Cost_Price!$C$18,"0.00")</f>
         <v>11.72 / 9.97</v>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Cost_Price</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Ex-showroom outright 2028 / 2035 (₹ lakh)</t>
         </is>
       </c>
-      <c r="B16" s="10" t="str">
+      <c r="B19" s="6" t="str">
         <f>TEXT(Cost_Price!$B$27,"0.00")&amp;" / "&amp;TEXT(Cost_Price!$C$27,"0.00")</f>
         <v>13.82 / 11.76</v>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Cost_Price</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Battery-EMI car price 2028 / 2035 (₹ lakh)</t>
         </is>
       </c>
-      <c r="B17" s="10" t="str">
+      <c r="B20" s="6" t="str">
         <f>TEXT(Cost_Price!$B$28,"0.00")&amp;" / "&amp;TEXT(Cost_Price!$C$28,"0.00")</f>
         <v>9.20 / 8.01</v>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Cost_Price</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Battery EMI 2028 / 2035 (₹/km) · break-even at 60k km</t>
         </is>
       </c>
-      <c r="B18" s="10" t="str">
+      <c r="B21" s="6" t="str">
         <f>TEXT(Inputs!$B$51,"0.0")&amp;" / "&amp;TEXT(Inputs!$B$52,"0.0")&amp;" · "&amp;TEXT(BaaS!$B$10,"0.00")&amp;" / "&amp;TEXT(BaaS!$C$10,"0.00")</f>
         <v>2.1 / 1.7 · 2.03 / 1.65</v>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>BaaS</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Price walk: chosen cost sits between Ertiga and e VITARA anchors</t>
         </is>
       </c>
-      <c r="B19" s="10" t="str">
+      <c r="B22" s="6" t="str">
         <f>Price_Walk!B34</f>
         <v>Yes</v>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Price_Walk</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>City range / at 70% SoH / Tour-e Long highway (km)</t>
         </is>
       </c>
-      <c r="B20" s="10" t="str">
-        <f>TEXT(BaaS!$B$27,"0")&amp;" / "&amp;TEXT(BaaS!$B$28,"0")&amp;" / "&amp;TEXT(BaaS!$B$33,"0")</f>
+      <c r="B23" s="6" t="str">
+        <f>TEXT(BaaS!$B$29,"0")&amp;" / "&amp;TEXT(BaaS!$B$30,"0")&amp;" / "&amp;TEXT(BaaS!$B$35,"0")</f>
         <v>307 / 215 / 317</v>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>BaaS</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>STRESS AND OUTLOOK</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>If the battery were leased (18% GST): owner-driver gain per month (₹)</t>
         </is>
       </c>
-      <c r="B22" s="8">
+      <c r="B25" s="8">
         <f>Sensitivity!E63</f>
         <v>3249.9999999999927</v>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Sensitivity H</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>CNG price at which Tour-e + EMI loses its edge, owner-driver (₹/kg)</t>
         </is>
       </c>
-      <c r="B23" s="8">
+      <c r="B26" s="8">
         <f>Sensitivity!E67</f>
         <v>64.39999999999999</v>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>Sensitivity G</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>2035: owner-driver gain per month, Tour-e + EMI (₹)</t>
         </is>
       </c>
-      <c r="B24" s="8">
+      <c r="B27" s="8">
         <f>Scenario_2035!C11</f>
         <v>10000.0</v>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Scenario_2035</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>WHY MARUTI</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Maruti programme payback year</t>
         </is>
       </c>
-      <c r="B25" s="6">
+      <c r="B29" s="10">
         <f>Maruti_Case!$B$16</f>
         <v>2033.0</v>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Maruti_Case</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Tour-e volume in 2031 vs Maruti's EV sales today (×)</t>
+        </is>
+      </c>
+      <c r="B30" s="9">
+        <f>Maruti_Case!$B$20</f>
+        <v>3.774154589371981</v>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Maruti_Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>How to use</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>1. Change any blue input on the Inputs sheet; every other sheet is formula-driven.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>2. Sheets: Inputs → Cost_Price → Price_Walk → BaaS → TCO → Driver_Economics → Fleet_Economics → Sensitivity → Scenario_2035 → Maruti_Case → Sources.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>3. Capital cost uses Excel PMT: annual loan payment at 10.5% over 5 years with the residual value as the loan's future value, plus 3% insurance on the full insured value.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>4. Tour-e is the fleet version of Maruti's YMC MPV on HEARTECT-e, using the e VITARA's 49 kWh (Tour-e) and 61 kWh (Tour-e Long) LFP packs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
-        <is>
-          <t>5. All values are in 2026 rupees with no inflation. Tour-e figures are design targets and team estimates, not current prices.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>6. Road-tax / permit waivers for EVs and any state purchase incentives are excluded, so the EV case is conservative.</t>
+          <t>1. Change any blue input on the Inputs sheet; every other sheet is formula-driven.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>2. Sheets: Inputs → Cost_Price → Price_Walk → BaaS → TCO → Driver_Economics → Fleet_Economics → Sensitivity → Scenario_2035 → Maruti_Case → Sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>3. Capital cost uses Excel PMT: annual loan payment at 10.5% over 5 years with the residual value as the loan's future value, plus 3% insurance on the full insured value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>4. Tour-e is the fleet version of Maruti's YMC MPV on HEARTECT-e, using the e VITARA's 49 kWh (Tour-e) and 61 kWh (Tour-e Long) LFP packs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>5. All values are in 2026 rupees with no inflation. Tour-e figures are design targets and team estimates, not current prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>6. Road-tax / permit waivers for EVs and any state purchase incentives are excluded, so the EV case is conservative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Colour key: blue on yellow = input; black = formula; green-tinted = headline output.</t>
         </is>
@@ -1532,15 +1607,15 @@
           <t>TOTAL (₹/km)</t>
         </is>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="6">
         <f>B5+B6+B7+B9</f>
         <v>10.09</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="6">
         <f>C5+C6+C7+C9</f>
         <v>8.09</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="6">
         <f>D5+D6+D7+D9</f>
         <v>8.03</v>
       </c>
@@ -1583,7 +1658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1985,35 +2060,35 @@
         </is>
       </c>
       <c r="B13" s="29" t="str">
-        <f>IF(B12&gt;=Inputs!$B$62,2028,"")</f>
+        <f>IF(B12&gt;=Inputs!$B$65,2028,"")</f>
         <v/>
       </c>
       <c r="C13" s="29" t="str">
-        <f>IF(C12&gt;=Inputs!$B$62,2029,"")</f>
+        <f>IF(C12&gt;=Inputs!$B$65,2029,"")</f>
         <v/>
       </c>
       <c r="D13" s="29" t="str">
-        <f>IF(D12&gt;=Inputs!$B$62,2030,"")</f>
+        <f>IF(D12&gt;=Inputs!$B$65,2030,"")</f>
         <v/>
       </c>
       <c r="E13" s="29" t="str">
-        <f>IF(E12&gt;=Inputs!$B$62,2031,"")</f>
+        <f>IF(E12&gt;=Inputs!$B$65,2031,"")</f>
         <v/>
       </c>
       <c r="F13" s="29" t="str">
-        <f>IF(F12&gt;=Inputs!$B$62,2032,"")</f>
+        <f>IF(F12&gt;=Inputs!$B$65,2032,"")</f>
         <v/>
       </c>
       <c r="G13" s="29">
-        <f>IF(G12&gt;=Inputs!$B$62,2033,"")</f>
+        <f>IF(G12&gt;=Inputs!$B$65,2033,"")</f>
         <v>2033.0</v>
       </c>
       <c r="H13" s="29">
-        <f>IF(H12&gt;=Inputs!$B$62,2034,"")</f>
+        <f>IF(H12&gt;=Inputs!$B$65,2034,"")</f>
         <v>2034.0</v>
       </c>
       <c r="I13" s="29">
-        <f>IF(I12&gt;=Inputs!$B$62,2035,"")</f>
+        <f>IF(I12&gt;=Inputs!$B$65,2035,"")</f>
         <v>2035.0</v>
       </c>
     </row>
@@ -2024,7 +2099,7 @@
         </is>
       </c>
       <c r="B15" s="8">
-        <f>Inputs!$B$62</f>
+        <f>Inputs!$B$65</f>
         <v>1500.0</v>
       </c>
     </row>
@@ -2034,7 +2109,7 @@
           <t>Payback year (capex fully recovered)</t>
         </is>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="10">
         <f>MIN(B13:I13)</f>
         <v>2033.0</v>
       </c>
@@ -2046,7 +2121,7 @@
         </is>
       </c>
       <c r="B17" s="8">
-        <f>Inputs!$B$62*100/Cost_Price!$B$17</f>
+        <f>Inputs!$B$65*100/Cost_Price!$B$17</f>
         <v>214285.7142857143</v>
       </c>
     </row>
@@ -2061,10 +2136,58 @@
         <v>3883.1914285714283</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>Maruti EV sales today, annualised (units)</t>
+        </is>
+      </c>
+      <c r="B19" s="8">
+        <f>Inputs!$B$63*12</f>
+        <v>13248.0</v>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Sep 2026 run-rate × 12.</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Not counted (upside): battery-EMI programme margin, FleetOS subscriptions, service and parts revenue, and compliance value of high-km EV sales under CAFE rules.</t>
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>Tour-e volume in 2031 vs Maruti's EV sales today</t>
+        </is>
+      </c>
+      <c r="B20" s="34">
+        <f>E5/B19</f>
+        <v>3.774154589371981</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Tour-e alone would multiply Maruti's EV volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>CAFE III credit-equivalent units in 2031</t>
+        </is>
+      </c>
+      <c r="B21" s="8">
+        <f>E5*Inputs!$B$64</f>
+        <v>150000.0</v>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Each battery EV counts 3× toward CAFE III compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Not counted (upside): battery-EMI programme margin, FleetOS subscriptions, driver-hub charging margin, service and parts revenue, and the CAFE III credit value.</t>
         </is>
       </c>
     </row>
@@ -2130,17 +2253,17 @@
       <c r="A5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="B5" s="35" t="inlineStr">
         <is>
           <t>Maruti Suzuki press release (Feb 2026)</t>
         </is>
       </c>
-      <c r="C5" s="34" t="inlineStr">
+      <c r="C5" s="35" t="inlineStr">
         <is>
           <t>e VITARA BaaS ₹10.99 L + ₹3.99/km; retail BaaS usage basis</t>
         </is>
       </c>
-      <c r="D5" s="35" t="inlineStr">
+      <c r="D5" s="36" t="inlineStr">
         <is>
           <t>https://www.marutisuzuki.com/corporate/media/press-releases/2026/february/india-goes-electric-with-maruti-suzuki-e-vitara-introductory-baas-price-starts</t>
         </is>
@@ -2150,17 +2273,17 @@
       <c r="A6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="34" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Autocar India – BaaS prices of e Vitara explained</t>
         </is>
       </c>
-      <c r="C6" s="34" t="inlineStr">
+      <c r="C6" s="35" t="inlineStr">
         <is>
           <t>Pack value ~₹5 L (49 kWh); 1,800 km/month minimum</t>
         </is>
       </c>
-      <c r="D6" s="35" t="inlineStr">
+      <c r="D6" s="36" t="inlineStr">
         <is>
           <t>https://www.autocarindia.com/auto-features/baas-prices-of-maruti-e-vitara-explained-440247</t>
         </is>
@@ -2170,17 +2293,17 @@
       <c r="A7" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="34" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>Autocar India – Maruti prices after GST cuts (Sep 2025)</t>
         </is>
       </c>
-      <c r="C7" s="34" t="inlineStr">
+      <c r="C7" s="35" t="inlineStr">
         <is>
           <t>Ertiga Tour M CNG post-GST ex-showroom</t>
         </is>
       </c>
-      <c r="D7" s="35" t="inlineStr">
+      <c r="D7" s="36" t="inlineStr">
         <is>
           <t>https://www.autocarindia.com/car-news-amp/maruti-suzuki-prices-after-gst-cuts-the-swift-gets-a-lakh-cheaper-437189</t>
         </is>
@@ -2190,17 +2313,17 @@
       <c r="A8" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="34" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>Outlook Business – Delhi CNG ₹86.98/kg</t>
         </is>
       </c>
-      <c r="C8" s="34" t="inlineStr">
+      <c r="C8" s="35" t="inlineStr">
         <is>
           <t>CNG price, Aug–Sep 2026</t>
         </is>
       </c>
-      <c r="D8" s="35" t="inlineStr">
+      <c r="D8" s="36" t="inlineStr">
         <is>
           <t>https://www.outlookbusiness.com/economy-and-policy/delhi-cng-to-cost-8698kg-as-igl-passes-on-rising-lng-costs</t>
         </is>
@@ -2210,17 +2333,17 @@
       <c r="A9" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="34" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>BloombergNEF – 2025 battery price survey</t>
         </is>
       </c>
-      <c r="C9" s="34" t="inlineStr">
+      <c r="C9" s="35" t="inlineStr">
         <is>
           <t>Pack prices: global $108/kWh; China $84/kWh; LFP $81/kWh</t>
         </is>
       </c>
-      <c r="D9" s="35" t="inlineStr">
+      <c r="D9" s="36" t="inlineStr">
         <is>
           <t>https://about.bnef.com/insights/clean-transport/lithium-ion-battery-pack-prices-fall-to-108-per-kilowatt-hour-despite-rising-metal-prices-bloombergnef/</t>
         </is>
@@ -2230,17 +2353,17 @@
       <c r="A10" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="34" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>ClearTax – GST on cars (GST 2.0)</t>
         </is>
       </c>
-      <c r="C10" s="34" t="inlineStr">
+      <c r="C10" s="35" t="inlineStr">
         <is>
           <t>EV 5%; &gt;4 m petrol/CNG 40%, from 22 Sep 2025</t>
         </is>
       </c>
-      <c r="D10" s="35" t="inlineStr">
+      <c r="D10" s="36" t="inlineStr">
         <is>
           <t>https://cleartax.in/s/gst-on-cars</t>
         </is>
@@ -2250,17 +2373,17 @@
       <c r="A11" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="34" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>CEEW (2025) – Cost of ownership for road transport</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
+      <c r="C11" s="35" t="inlineStr">
         <is>
           <t>EVs cheapest-to-own taxi option; CNG next</t>
         </is>
       </c>
-      <c r="D11" s="35" t="inlineStr">
+      <c r="D11" s="36" t="inlineStr">
         <is>
           <t>https://www.ceew.in/publications/cost-of-ownership-for-road-transport-sector-for-different-vehicle-segments-fuels-and-powertrains</t>
         </is>
@@ -2270,17 +2393,17 @@
       <c r="A12" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="34" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>MeraEV – EV charging cost in India (2026)</t>
         </is>
       </c>
-      <c r="C12" s="34" t="inlineStr">
+      <c r="C12" s="35" t="inlineStr">
         <is>
           <t>Public DC tariff range</t>
         </is>
       </c>
-      <c r="D12" s="35" t="inlineStr">
+      <c r="D12" s="36" t="inlineStr">
         <is>
           <t>https://www.meraev.com/blog/ev-charging-cost-in-india-full-guide</t>
         </is>
@@ -2290,17 +2413,17 @@
       <c r="A13" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="34" t="inlineStr">
+      <c r="B13" s="35" t="inlineStr">
         <is>
           <t>MyMotor – state-wise EV charging tariffs</t>
         </is>
       </c>
-      <c r="C13" s="34" t="inlineStr">
+      <c r="C13" s="35" t="inlineStr">
         <is>
           <t>Depot / EV tariff range</t>
         </is>
       </c>
-      <c r="D13" s="35" t="inlineStr">
+      <c r="D13" s="36" t="inlineStr">
         <is>
           <t>https://www.mymotor.in/blog/ev-charging-cost-india-state-wise-tariff</t>
         </is>
@@ -2310,17 +2433,17 @@
       <c r="A14" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="34" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>HDFC Sky – INR/USD daily reports (Jun–Aug 2026)</t>
         </is>
       </c>
-      <c r="C14" s="34" t="inlineStr">
+      <c r="C14" s="35" t="inlineStr">
         <is>
           <t>Exchange rate ~₹95/$</t>
         </is>
       </c>
-      <c r="D14" s="35" t="inlineStr">
+      <c r="D14" s="36" t="inlineStr">
         <is>
           <t>https://hdfcsky.com/news/inr-usd-rate-august-11-2026-rupee-falls-95-43</t>
         </is>
@@ -2330,17 +2453,17 @@
       <c r="A15" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="34" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>Rushlane – Ertiga CNG launch</t>
         </is>
       </c>
-      <c r="C15" s="34" t="inlineStr">
+      <c r="C15" s="35" t="inlineStr">
         <is>
           <t>Claimed 26.11 km/kg CNG efficiency</t>
         </is>
       </c>
-      <c r="D15" s="35" t="inlineStr">
+      <c r="D15" s="36" t="inlineStr">
         <is>
           <t>https://www.rushlane.com/2019-maruti-ertiga-cng-launched-12318513.html</t>
         </is>
@@ -2350,17 +2473,17 @@
       <c r="A16" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="34" t="inlineStr">
+      <c r="B16" s="35" t="inlineStr">
         <is>
           <t>Business Standard – e VITARA pricing and BaaS (Feb 2026)</t>
         </is>
       </c>
-      <c r="C16" s="34" t="inlineStr">
+      <c r="C16" s="35" t="inlineStr">
         <is>
           <t>BaaS structured as a dual loan (vehicle + battery)</t>
         </is>
       </c>
-      <c r="D16" s="35" t="inlineStr">
+      <c r="D16" s="36" t="inlineStr">
         <is>
           <t>https://www.business-standard.com/industry/auto/maruti-suzuki-enters-ev-market-with-sharp-e-vitara-pricing-baas-model-126021700866_1.html</t>
         </is>
@@ -2370,17 +2493,17 @@
       <c r="A17" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="34" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>Cartoq – Maruti YMC electric MPV</t>
         </is>
       </c>
-      <c r="C17" s="34" t="inlineStr">
+      <c r="C17" s="35" t="inlineStr">
         <is>
           <t>YMC on HEARTECT-e; expected to use the 49 / 61 kWh packs (media reports)</t>
         </is>
       </c>
-      <c r="D17" s="35" t="inlineStr">
+      <c r="D17" s="36" t="inlineStr">
         <is>
           <t>https://www.cartoq.com/car-news/maruti-suzuki-ymc-electric-mpv-launch-2026/</t>
         </is>
@@ -2390,17 +2513,17 @@
       <c r="A18" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="34" t="inlineStr">
+      <c r="B18" s="35" t="inlineStr">
         <is>
           <t>CarDekho – e VITARA Delta specifications</t>
         </is>
       </c>
-      <c r="C18" s="34" t="inlineStr">
+      <c r="C18" s="35" t="inlineStr">
         <is>
           <t>~45 min 10–80% DC (50 kW); 7.4 kW AC on-board charger</t>
         </is>
       </c>
-      <c r="D18" s="35" t="inlineStr">
+      <c r="D18" s="36" t="inlineStr">
         <is>
           <t>https://www.cardekho.com/overview/Maruti_e_Vitara/Maruti_e_Vitara_Delta.htm</t>
         </is>
@@ -2435,7 +2558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3619,11 +3742,11 @@
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>Retail e VITARA BaaS rate (benchmark)</t>
+          <t>Battery EMI for fleets contracting 80,000 km/yr (2028)</t>
         </is>
       </c>
       <c r="B53" s="17" t="n">
-        <v>3.99</v>
+        <v>1.7</v>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
@@ -3632,73 +3755,73 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Sourced</t>
+          <t>Team decision</t>
         </is>
       </c>
       <c r="E53" s="14" t="inlineStr">
         <is>
-          <t>Maruti Suzuki press release, Feb 2026 (49 kWh pack).</t>
+          <t>Usage-tiered pricing: the same battery spread over more contracted km. Rounded up from the 80,000 km break-even on the BaaS sheet.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>Retail e VITARA BaaS usage basis</t>
-        </is>
-      </c>
-      <c r="B54" s="13" t="n">
-        <v>21900</v>
+          <t>Retail e VITARA BaaS rate (benchmark)</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="n">
+        <v>3.99</v>
       </c>
       <c r="C54" s="12" t="inlineStr">
         <is>
-          <t>km/yr</t>
+          <t>₹/km</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Sourced (derived)</t>
+          <t>Sourced</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
         <is>
-          <t>Rate is quoted on ~60 km/day (Maruti minimum 1,800 km/month); 60 × 365 = 21,900.</t>
+          <t>Maruti Suzuki press release, Feb 2026 (49 kWh pack).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>e VITARA Delta (49 kWh) ex-showroom: BaaS price</t>
-        </is>
-      </c>
-      <c r="B55" s="17" t="n">
-        <v>10.99</v>
+          <t>Retail e VITARA BaaS usage basis</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="n">
+        <v>21900</v>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>₹ lakh</t>
+          <t>km/yr</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Sourced</t>
+          <t>Sourced (derived)</t>
         </is>
       </c>
       <c r="E55" s="14" t="inlineStr">
         <is>
-          <t>Maruti Suzuki, Feb 2026.</t>
+          <t>Rate is quoted on ~60 km/day (Maruti minimum 1,800 km/month); 60 × 365 = 21,900.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>e VITARA Delta (49 kWh) ex-showroom: with battery</t>
+          <t>e VITARA Delta (49 kWh) ex-showroom: BaaS price</t>
         </is>
       </c>
       <c r="B56" s="17" t="n">
-        <v>15.99</v>
+        <v>10.99</v>
       </c>
       <c r="C56" s="12" t="inlineStr">
         <is>
@@ -3712,127 +3835,202 @@
       </c>
       <c r="E56" s="14" t="inlineStr">
         <is>
-          <t>Autocar India / Upstox, Feb 2026.</t>
+          <t>Maruti Suzuki, Feb 2026.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
+          <t>e VITARA Delta (49 kWh) ex-showroom: with battery</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="n">
+        <v>15.99</v>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>₹ lakh</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>Autocar India / Upstox, Feb 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
           <t>Nexa retail dealer margin (for the e VITARA walk)</t>
         </is>
       </c>
-      <c r="B57" s="15" t="n">
+      <c r="B58" s="15" t="n">
         <v>0.05</v>
       </c>
-      <c r="C57" s="12" t="inlineStr">
+      <c r="C58" s="12" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D58" s="7" t="inlineStr">
         <is>
           <t>Team assumption</t>
         </is>
       </c>
-      <c r="E57" s="14" t="inlineStr">
+      <c r="E58" s="14" t="inlineStr">
         <is>
           <t>Retail (Nexa) margins are higher than fleet margins.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>6 · Driver revenue (illustrative only)</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n"/>
-      <c r="C58" s="5" t="n"/>
-      <c r="D58" s="5" t="n"/>
-      <c r="E58" s="5" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="12" t="inlineStr">
-        <is>
-          <t>Net fare earnings to driver per km driven</t>
-        </is>
-      </c>
-      <c r="B59" s="17" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>₹/km</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>Team assumption</t>
-        </is>
-      </c>
-      <c r="E59" s="14" t="inlineStr">
-        <is>
-          <t>After platform commission and dead km. ONLY used for absolute income; the Tour-e uplift does not depend on it.</t>
-        </is>
-      </c>
+      <c r="B59" s="5" t="n"/>
+      <c r="C59" s="5" t="n"/>
+      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
         <is>
+          <t>Net fare earnings to driver per km driven</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>₹/km</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Team assumption</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
+        <is>
+          <t>After platform commission and dead km. ONLY used for absolute income; the Tour-e uplift does not depend on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
           <t>Example fleet size</t>
         </is>
       </c>
-      <c r="B60" s="13" t="n">
+      <c r="B61" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="C60" s="12" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>cars</t>
         </is>
       </c>
-      <c r="D60" s="7" t="inlineStr">
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>Illustrative</t>
         </is>
       </c>
-      <c r="E60" s="14" t="inlineStr">
+      <c r="E61" s="14" t="inlineStr">
         <is>
           <t>For fleet-level totals.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>7 · Maruti programme</t>
         </is>
       </c>
-      <c r="B61" s="5" t="n"/>
-      <c r="C61" s="5" t="n"/>
-      <c r="D61" s="5" t="n"/>
-      <c r="E61" s="5" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="12" t="inlineStr">
+      <c r="B62" s="5" t="n"/>
+      <c r="C62" s="5" t="n"/>
+      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="5" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>Maruti EV sales, September 2026</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="n">
+        <v>1104</v>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>units/month</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>Vahan registrations, Sep 2026 (Autopunditz / Rushlane); about 3% of India's EV car market, vs Tata ~42%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>CAFE III super-credit multiplier for battery EVs</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E64" s="14" t="inlineStr">
+        <is>
+          <t>CAFE III notified for 1 Apr 2027 – 31 Mar 2032: BEVs count 3× (Autocar India / Autocar Professional).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t>Tour-e programme capex (derivative of YMC)</t>
         </is>
       </c>
-      <c r="B62" s="13" t="n">
+      <c r="B65" s="13" t="n">
         <v>1500</v>
       </c>
-      <c r="C62" s="12" t="inlineStr">
+      <c r="C65" s="12" t="inlineStr">
         <is>
           <t>₹ crore</t>
         </is>
       </c>
-      <c r="D62" s="7" t="inlineStr">
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>Team assumption</t>
         </is>
       </c>
-      <c r="E62" s="14" t="inlineStr">
+      <c r="E65" s="14" t="inlineStr">
         <is>
           <t>Body-side and sliding-door tooling, taxi trims, validation, FleetOS and BaaS set-up. Lower than a new platform because YMC carries the HEARTECT-e cost.</t>
         </is>
@@ -4196,11 +4394,11 @@
           <t>Ex-factory cost (total)</t>
         </is>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="6">
         <f>SUM(B5:B17)</f>
         <v>11.719999999999999</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="6">
         <f>SUM(C5:C17)</f>
         <v>9.975</v>
       </c>
@@ -4367,11 +4565,11 @@
           <t>Ex-showroom price, bought outright (₹ L)</t>
         </is>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="6">
         <f>B18*B26</f>
         <v>13.8220992</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="6">
         <f>C18*C26</f>
         <v>11.764116000000001</v>
       </c>
@@ -4391,11 +4589,11 @@
           <t>Fleet BaaS: vehicle-only price (₹ L)</t>
         </is>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="6">
         <f>B20*B26</f>
         <v>9.199008000000001</v>
       </c>
-      <c r="C28" s="10">
+      <c r="C28" s="6">
         <f>C20*C26</f>
         <v>8.0078544</v>
       </c>
@@ -4771,7 +4969,7 @@
           <t>→ Anchor A: Tour-e non-battery cost</t>
         </is>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="6">
         <f>B13+SUM(B14:B19)</f>
         <v>7.78315527065527</v>
       </c>
@@ -4797,7 +4995,7 @@
         </is>
       </c>
       <c r="B23" s="18">
-        <f>Inputs!$B$55</f>
+        <f>Inputs!$B$56</f>
         <v>10.99</v>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -4825,7 +5023,7 @@
         </is>
       </c>
       <c r="B25" s="18">
-        <f>B24/(1+Inputs!$B$57)</f>
+        <f>B24/(1+Inputs!$B$58)</f>
         <v>9.968253968253968</v>
       </c>
       <c r="C25" s="7" t="inlineStr"/>
@@ -4889,7 +5087,7 @@
           <t>→ Anchor B: Tour-e non-battery cost</t>
         </is>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="6">
         <f>B26+SUM(B27:B29)</f>
         <v>8.229864785420341</v>
       </c>
@@ -4914,7 +5112,7 @@
           <t>Chosen non-battery cost (Cost_Price stack)</t>
         </is>
       </c>
-      <c r="B33" s="10">
+      <c r="B33" s="6">
         <f>Cost_Price!$B$20</f>
         <v>7.799999999999999</v>
       </c>
@@ -4947,7 +5145,7 @@
         </is>
       </c>
       <c r="B35" s="18">
-        <f>Cost_Price!$B$27-Inputs!$B$56</f>
+        <f>Cost_Price!$B$27-Inputs!$B$57</f>
         <v>-2.1679008</v>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -4963,7 +5161,7 @@
         </is>
       </c>
       <c r="B36" s="18">
-        <f>Cost_Price!$B$28-Inputs!$B$55</f>
+        <f>Cost_Price!$B$28-Inputs!$B$56</f>
         <v>-1.7909919999999993</v>
       </c>
       <c r="C36" s="7" t="inlineStr"/>
@@ -4975,7 +5173,7 @@
         </is>
       </c>
       <c r="B37" s="18">
-        <f>Inputs!$B$56-Inputs!$B$55</f>
+        <f>Inputs!$B$57-Inputs!$B$56</f>
         <v>5.0</v>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -5013,7 +5211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -5144,11 +5342,11 @@
           <t>Annual EMI revenue required (₹ L/yr)</t>
         </is>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="6">
         <f>B6+B7+B8</f>
         <v>1.2168871574623759</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="6">
         <f>C6+C7+C8</f>
         <v>0.9887208154381802</v>
       </c>
@@ -5160,11 +5358,11 @@
           <t>Break-even at minimum contract km (₹/km)</t>
         </is>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="6">
         <f>B9*100000/Inputs!$B$50</f>
         <v>2.028145262437293</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="6">
         <f>C9*100000/Inputs!$B$50</f>
         <v>1.6478680257303004</v>
       </c>
@@ -5200,11 +5398,11 @@
           <t>Chosen fleet battery EMI (₹/km)</t>
         </is>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="6">
         <f>Inputs!$B$51</f>
         <v>2.1</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="6">
         <f>Inputs!$B$52</f>
         <v>1.7</v>
       </c>
@@ -5274,255 +5472,289 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Fleet tier: battery EMI for 80,000 km contracts (₹/km)</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>Inputs!$B$53</f>
+        <v>1.7</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Headroom over the 80,000 km break-even shown next.</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Headroom over the 80,000 km break-even</t>
+        </is>
+      </c>
+      <c r="B17" s="26">
+        <f>B16/B11-1</f>
+        <v>0.11760568074040911</v>
+      </c>
+      <c r="C17" s="26" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Must be ≥ 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Why the fleet rate is half the retail e VITARA rate</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Retail e VITARA BaaS (₹/km)</t>
-        </is>
-      </c>
-      <c r="B18" s="18">
-        <f>Inputs!$B$53</f>
-        <v>3.99</v>
-      </c>
-      <c r="C18" s="18" t="inlineStr"/>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>Maruti Suzuki, Feb 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Retail usage basis (km/yr)</t>
-        </is>
-      </c>
-      <c r="B19" s="27">
-        <f>Inputs!$B$54</f>
-        <v>21900.0</v>
-      </c>
-      <c r="C19" s="27" t="inlineStr"/>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>~60 km/day.</t>
-        </is>
-      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>Fleet minimum km ÷ retail km</t>
-        </is>
-      </c>
-      <c r="B20" s="28">
-        <f>Inputs!$B$50/Inputs!$B$54</f>
-        <v>2.73972602739726</v>
-      </c>
-      <c r="C20" s="28" t="inlineStr"/>
+          <t>Retail e VITARA BaaS (₹/km)</t>
+        </is>
+      </c>
+      <c r="B20" s="18">
+        <f>Inputs!$B$54</f>
+        <v>3.99</v>
+      </c>
+      <c r="C20" s="18" t="inlineStr"/>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Same pack, ~2.7× the km → far lower ₹/km.</t>
+          <t>Maruti Suzuki, Feb 2026.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
+          <t>Retail usage basis (km/yr)</t>
+        </is>
+      </c>
+      <c r="B21" s="27">
+        <f>Inputs!$B$55</f>
+        <v>21900.0</v>
+      </c>
+      <c r="C21" s="27" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>~60 km/day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Fleet minimum km ÷ retail km</t>
+        </is>
+      </c>
+      <c r="B22" s="28">
+        <f>Inputs!$B$50/Inputs!$B$55</f>
+        <v>2.73972602739726</v>
+      </c>
+      <c r="C22" s="28" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Same pack, ~2.7× the km → far lower ₹/km.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
           <t>Retail rate spread over fleet km (₹/km)</t>
         </is>
       </c>
-      <c r="B21" s="18">
-        <f>Inputs!$B$53*Inputs!$B$54/Inputs!$B$50</f>
+      <c r="B23" s="18">
+        <f>Inputs!$B$54*Inputs!$B$55/Inputs!$B$50</f>
         <v>1.45635</v>
       </c>
-      <c r="C21" s="18" t="inlineStr"/>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr"/>
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Pure scaling of the retail rate. The fleet EMI sits above this, so it is conservative for the programme.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Battery duty check</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Lifetime km at fleet duty (5 yrs)</t>
         </is>
       </c>
-      <c r="B24" s="27">
+      <c r="B26" s="27">
         <f>Inputs!$B$8*Inputs!$B$6</f>
         <v>400000.0</v>
       </c>
-      <c r="C24" s="27" t="inlineStr"/>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>4 lakh km design life.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Energy throughput at battery (kWh)</t>
-        </is>
-      </c>
-      <c r="B25" s="27">
-        <f>B24*Inputs!$B$20</f>
-        <v>60000.0</v>
-      </c>
-      <c r="C25" s="27" t="inlineStr"/>
-      <c r="D25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Equivalent full cycles (usable kWh)</t>
-        </is>
-      </c>
-      <c r="B26" s="27">
-        <f>B25/Inputs!$B$18</f>
-        <v>1304.3478260869565</v>
-      </c>
       <c r="C26" s="27" t="inlineStr"/>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>≈1,300–1,450 equivalent full cycles over 5 years – well within LFP cycle life (automotive LFP cells are typically rated 3,000+ cycles).</t>
+          <t>4 lakh km design life.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
+          <t>Energy throughput at battery (kWh)</t>
+        </is>
+      </c>
+      <c r="B27" s="27">
+        <f>B26*Inputs!$B$20</f>
+        <v>60000.0</v>
+      </c>
+      <c r="C27" s="27" t="inlineStr"/>
+      <c r="D27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Equivalent full cycles (usable kWh)</t>
+        </is>
+      </c>
+      <c r="B28" s="27">
+        <f>B27/Inputs!$B$18</f>
+        <v>1304.3478260869565</v>
+      </c>
+      <c r="C28" s="27" t="inlineStr"/>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>≈1,300–1,450 equivalent full cycles over 5 years – well within LFP cycle life (automotive LFP cells are typically rated 3,000+ cycles).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
           <t>Real-world city range (km)</t>
         </is>
       </c>
-      <c r="B27" s="29">
+      <c r="B29" s="29">
         <f>Inputs!$B$18/Inputs!$B$20</f>
         <v>306.6666666666667</v>
       </c>
-      <c r="C27" s="29" t="inlineStr"/>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="C29" s="29" t="inlineStr"/>
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>46 kWh usable ÷ 150 Wh/km.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Range at 70% SoH end-of-life (km)</t>
         </is>
       </c>
-      <c r="B28" s="29">
+      <c r="B30" s="29">
         <f>Inputs!$B$18*0.7/Inputs!$B$20</f>
         <v>214.66666666666666</v>
       </c>
-      <c r="C28" s="29" t="inlineStr"/>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="C30" s="29" t="inlineStr"/>
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Still covers a 200 km owner-driver day.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>Fleet day (km)</t>
         </is>
       </c>
-      <c r="B29" s="29">
+      <c r="B31" s="29">
         <f>Inputs!$B$8/Inputs!$B$10</f>
         <v>250.0</v>
       </c>
-      <c r="C29" s="29" t="inlineStr"/>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>80,000 km ÷ 320 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Shortfall at end of life, fleet day (km)</t>
-        </is>
-      </c>
-      <c r="B30" s="29">
-        <f>MAX(0,B29-B28)</f>
-        <v>35.33333333333334</v>
-      </c>
-      <c r="C30" s="29" t="inlineStr"/>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Covered by one DC top-up a day from about year 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>Km per day already budgeted on public DC (fleet)</t>
-        </is>
-      </c>
-      <c r="B31" s="29">
-        <f>(1-Inputs!$B$26)*B29</f>
-        <v>49.999999999999986</v>
-      </c>
       <c r="C31" s="29" t="inlineStr"/>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>The 20% DC share in the TCO already pays for this top-up, so no extra cost.</t>
+          <t>80,000 km ÷ 320 days.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
+          <t>Shortfall at end of life, fleet day (km)</t>
+        </is>
+      </c>
+      <c r="B32" s="29">
+        <f>MAX(0,B31-B30)</f>
+        <v>35.33333333333334</v>
+      </c>
+      <c r="C32" s="29" t="inlineStr"/>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Covered by one DC top-up a day from about year 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Km per day already budgeted on public DC (fleet)</t>
+        </is>
+      </c>
+      <c r="B33" s="29">
+        <f>(1-Inputs!$B$26)*B31</f>
+        <v>49.999999999999986</v>
+      </c>
+      <c r="C33" s="29" t="inlineStr"/>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>The 20% DC share in the TCO already pays for this top-up, so no extra cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
           <t>Tour-e Long range, city (km)</t>
         </is>
       </c>
-      <c r="B32" s="29">
+      <c r="B34" s="29">
         <f>Inputs!$B$19/Inputs!$B$20</f>
         <v>380.0</v>
       </c>
-      <c r="C32" s="29" t="inlineStr"/>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="C34" s="29" t="inlineStr"/>
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>61 kWh pack, 57 kWh usable.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Tour-e Long range, highway at ~100 km/h (km)</t>
         </is>
       </c>
-      <c r="B33" s="29">
+      <c r="B35" s="29">
         <f>Inputs!$B$19/Inputs!$B$21</f>
         <v>316.6666666666667</v>
       </c>
-      <c r="C33" s="29" t="inlineStr"/>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="C35" s="29" t="inlineStr"/>
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Covers 280–300 km corridors (e.g. Delhi–Jaipur) one way; top up before the return leg.</t>
         </is>
@@ -5671,7 +5903,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Fleet battery EMI, 2028 (a loan, so no GST on it).</t>
+          <t>Battery EMI, 2028, tiered by contracted km (a loan, so no GST on it).</t>
         </is>
       </c>
     </row>
@@ -5801,15 +6033,15 @@
           <t>TOTAL COST PER KM (₹/km)</t>
         </is>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="6">
         <f>B6+B7+B8+B13</f>
         <v>10.09</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="6">
         <f>C6+C7+C8+C13</f>
         <v>9.059999999999999</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="6">
         <f>D6+D7+D8+D13</f>
         <v>8.969999999999999</v>
       </c>
@@ -6004,8 +6236,8 @@
         <v>0.0</v>
       </c>
       <c r="C24" s="18">
-        <f>Inputs!$B$51</f>
-        <v>2.1</v>
+        <f>Inputs!$B$53</f>
+        <v>1.7</v>
       </c>
       <c r="D24" s="18">
         <f>0</f>
@@ -6013,7 +6245,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Fleet battery EMI, 2028 (a loan, so no GST on it).</t>
+          <t>Battery EMI, 2028, tiered by contracted km (a loan, so no GST on it).</t>
         </is>
       </c>
     </row>
@@ -6143,15 +6375,15 @@
           <t>TOTAL COST PER KM (₹/km)</t>
         </is>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="6">
         <f>B22+B23+B24+B29</f>
         <v>8.86</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C30" s="6">
         <f>C22+C23+C24+C29</f>
-        <v>7.7299999999999995</v>
-      </c>
-      <c r="D30" s="10">
+        <v>7.33</v>
+      </c>
+      <c r="D30" s="6">
         <f>D22+D23+D24+D29</f>
         <v>7.13</v>
       </c>
@@ -6173,7 +6405,7 @@
       </c>
       <c r="C31" s="18">
         <f>C30*Inputs!$B$8/100000</f>
-        <v>6.184</v>
+        <v>5.864</v>
       </c>
       <c r="D31" s="18">
         <f>D30*Inputs!$B$8/100000</f>
@@ -6197,7 +6429,7 @@
       </c>
       <c r="C32" s="18">
         <f>C31*Inputs!$B$6</f>
-        <v>30.92</v>
+        <v>29.32</v>
       </c>
       <c r="D32" s="18">
         <f>D31*Inputs!$B$6</f>
@@ -6221,7 +6453,7 @@
       </c>
       <c r="C33" s="18">
         <f>$B30-C30</f>
-        <v>1.13</v>
+        <v>1.5299999999999994</v>
       </c>
       <c r="D33" s="18">
         <f>$B30-D30</f>
@@ -6241,7 +6473,7 @@
       </c>
       <c r="C34" s="18">
         <f>C33*Inputs!$B$8/100000</f>
-        <v>0.9039999999999998</v>
+        <v>1.2239999999999993</v>
       </c>
       <c r="D34" s="18">
         <f>D33*Inputs!$B$8/100000</f>
@@ -6441,15 +6673,15 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>Inputs!$B$59*Inputs!$B$7/12</f>
+        <f>Inputs!$B$60*Inputs!$B$7/12</f>
         <v>67500.0</v>
       </c>
       <c r="C9" s="27">
-        <f>Inputs!$B$59*Inputs!$B$7/12</f>
+        <f>Inputs!$B$60*Inputs!$B$7/12</f>
         <v>67500.0</v>
       </c>
       <c r="D9" s="27">
-        <f>Inputs!$B$59*Inputs!$B$7/12</f>
+        <f>Inputs!$B$60*Inputs!$B$7/12</f>
         <v>67500.0</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -6588,7 +6820,7 @@
         </is>
       </c>
       <c r="B17" s="29">
-        <f>BaaS!$B$27</f>
+        <f>BaaS!$B$29</f>
         <v>306.6666666666667</v>
       </c>
     </row>
@@ -6706,15 +6938,15 @@
           <t>Maruti driver hub (base): 80% @ ₹11, 20% DC</t>
         </is>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="6">
         <f>(Inputs!$B$27*Inputs!$B$24+(1-Inputs!$B$27)*Inputs!$B$25)</f>
         <v>12.8</v>
       </c>
-      <c r="C27" s="10">
+      <c r="C27" s="6">
         <f>ROUND(Inputs!$B$20/Inputs!$B$22*(Inputs!$B$27*Inputs!$B$24+(1-Inputs!$B$27)*Inputs!$B$25),2)+Inputs!$B$29+Inputs!$B$51+TCO!C13</f>
         <v>9.059999999999999</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="6">
         <f>ROUND(Inputs!$B$20/Inputs!$B$22*(Inputs!$B$27*Inputs!$B$24+(1-Inputs!$B$27)*Inputs!$B$25),2)+Inputs!$B$29+TCO!D13</f>
         <v>8.969999999999999</v>
       </c>
@@ -6825,7 +7057,7 @@
       </c>
       <c r="C5" s="18">
         <f>TCO!C30</f>
-        <v>7.7299999999999995</v>
+        <v>7.33</v>
       </c>
       <c r="D5" s="18">
         <f>TCO!D30</f>
@@ -6849,7 +7081,7 @@
       </c>
       <c r="C6" s="18">
         <f>TCO!C31</f>
-        <v>6.184</v>
+        <v>5.864</v>
       </c>
       <c r="D6" s="18">
         <f>TCO!D31</f>
@@ -6863,15 +7095,15 @@
           <t>Annual saving per car vs CNG (₹ lakh)</t>
         </is>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="6">
         <f>TCO!B34</f>
         <v>0.0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="6">
         <f>TCO!C34</f>
-        <v>0.9039999999999998</v>
-      </c>
-      <c r="D7" s="10">
+        <v>1.2239999999999993</v>
+      </c>
+      <c r="D7" s="6">
         <f>TCO!D34</f>
         <v>1.3839999999999997</v>
       </c>
@@ -6893,7 +7125,7 @@
       </c>
       <c r="C8" s="18">
         <f>C7*Inputs!$B$6</f>
-        <v>4.519999999999999</v>
+        <v>6.1199999999999966</v>
       </c>
       <c r="D8" s="18">
         <f>D7*Inputs!$B$6</f>
@@ -6957,7 +7189,7 @@
       </c>
       <c r="C11" s="18">
         <f>((TCO!$B22+TCO!$B23)-(TCO!C22+TCO!C23+TCO!C24))*Inputs!$B$8/100000</f>
-        <v>0.5440000000000005</v>
+        <v>0.864</v>
       </c>
       <c r="D11" s="18">
         <f>((TCO!$B22+TCO!$B23)-(TCO!D22+TCO!D23+TCO!D24))*Inputs!$B$8/100000</f>
@@ -7000,15 +7232,15 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>B7*Inputs!$B$60/100</f>
+        <f>B7*Inputs!$B$61/100</f>
         <v>0.0</v>
       </c>
       <c r="C13" s="18">
-        <f>C7*Inputs!$B$60/100</f>
-        <v>0.9039999999999998</v>
+        <f>C7*Inputs!$B$61/100</f>
+        <v>1.2239999999999993</v>
       </c>
       <c r="D13" s="18">
-        <f>D7*Inputs!$B$60/100</f>
+        <f>D7*Inputs!$B$61/100</f>
         <v>1.3839999999999997</v>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -7024,15 +7256,15 @@
         </is>
       </c>
       <c r="B14" s="23">
-        <f>B9*Inputs!$B$60/100</f>
+        <f>B9*Inputs!$B$61/100</f>
         <v>10.745</v>
       </c>
       <c r="C14" s="23">
-        <f>C9*Inputs!$B$60/100</f>
+        <f>C9*Inputs!$B$61/100</f>
         <v>9.199008000000001</v>
       </c>
       <c r="D14" s="23">
-        <f>D9*Inputs!$B$60/100</f>
+        <f>D9*Inputs!$B$61/100</f>
         <v>13.8220992</v>
       </c>
       <c r="E14" s="7" t="inlineStr"/>
@@ -8083,7 +8315,7 @@
           <t>Battery EMI at which Tour-e = CNG (₹/km)</t>
         </is>
       </c>
-      <c r="E69" s="10">
+      <c r="E69" s="6">
         <f>(ROUND(Inputs!$B$32/Inputs!$B$33,2)+Inputs!$B$34+ROUND((PMT(Inputs!$B$11,Inputs!$B$6,-Inputs!$B$31,Inputs!$B$13*Inputs!$B$31)+Inputs!$B$12*Inputs!$B$31)*100000/Inputs!$B$7,2))-ROUND(Inputs!$B$20/Inputs!$B$22*(Inputs!$B$27*Inputs!$B$24+(1-Inputs!$B$27)*Inputs!$B$25),2)-Inputs!$B$29-ROUND((PMT(Inputs!$B$11,Inputs!$B$6,-Cost_Price!$B$28,Inputs!$B$15*Cost_Price!$B$28)+Inputs!$B$12*Cost_Price!$B$28+Inputs!$B$12*Cost_Price!$B$29)*100000/Inputs!$B$7,2)</f>
         <v>3.13</v>
       </c>

</xml_diff>